<commit_message>
adding total row at the end of the csvs
</commit_message>
<xml_diff>
--- a/World Bank Documents PAD/PID/Pivot Tables New/livestock_pivot_tables.xlsx
+++ b/World Bank Documents PAD/PID/Pivot Tables New/livestock_pivot_tables.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M117"/>
+  <dimension ref="A1:M118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5808,6 +5808,49 @@
         <v>1</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="D118" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E118" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G118" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="I118" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="J118" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K118" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="L118" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="M118" s="3" t="n">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5819,7 +5862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8766,6 +8809,31 @@
       </c>
       <c r="G117" s="3" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="D118" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="E118" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="G118" s="3" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>